<commit_message>
Régénérer l'historique CSV à chaque exécution : un point par date de terrain
L'export ajoutait une ligne par lancement du script, datée du sondage le
plus récent : plusieurs lancements le même jour créaient des doublons, et
plusieurs sondages saisis d'un coup ne produisaient qu'un seul point.

Le calcul est extrait dans calculer_moyennes(sondages, date_ref) et le
CSV est désormais entièrement reconstruit : pour chaque date de fin de
terrain distincte, moyenne pondérée des sondages connus à cette date,
fraîcheur mesurée depuis cette date. Le script est idempotent et la date
d'exécution n'a plus d'influence sur le fichier.

Mise à jour du classeur de sondages (nouveaux sondages saisis).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012cuMa5M8ynMEEJU6YTHSxt
</commit_message>
<xml_diff>
--- a/sondages_2027.xlsx
+++ b/sondages_2027.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Desktop/Infographies/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Projets/agregateur-sondages-2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A791B33-83A3-2A40-83D9-8A43BA9C2402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F8FB31-A090-B445-ABDD-387BF9632EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="500" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T1 — intentions de vote" sheetId="1" r:id="rId1"/>
     <sheet name="T2 — hypothèses (référence)" sheetId="2" r:id="rId2"/>
     <sheet name="T1 — scénarios alternatifs" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="89">
   <si>
     <t>Institut</t>
   </si>
@@ -133,9 +133,6 @@
     <t>Attal ET Le Pen (deux axes, p.11). Centre = Attal, RN = Le Pen. Hors blocs : Arthaud 0,5 ; Roussel 3 ; Villepin 3 ; NDA 2</t>
   </si>
   <si>
-    <t>RN : Bardella ; PS : Glucksmann ; centre : Philippe ; gauche désunie. Réf. = hypothèse Philippe seul (p.7). Hors blocs : Arthaud 0,5 ; Roussel 3,5 ; Villepin 2,5 ; NDA 2</t>
-  </si>
-  <si>
     <t>Ipsos</t>
   </si>
   <si>
@@ -145,9 +142,6 @@
     <t>Hollande+Philippe+Bardella</t>
   </si>
   <si>
-    <t>Glicksman+Attal+philippe+Le Pen</t>
-  </si>
-  <si>
     <t>Attal+Bardella</t>
   </si>
   <si>
@@ -155,6 +149,147 @@
   </si>
   <si>
     <t>Attal+Le Pen</t>
+  </si>
+  <si>
+    <t>OpinionWay</t>
+  </si>
+  <si>
+    <t>RN : indifférent ; PS : Glucksmann</t>
+  </si>
+  <si>
+    <t>Attal</t>
+  </si>
+  <si>
+    <t>Attal et n'importe qui pour RN</t>
+  </si>
+  <si>
+    <t>NSP : 27,4 % !!</t>
+  </si>
+  <si>
+    <t>Le Pen vs Edouard Philippe</t>
+  </si>
+  <si>
+    <t>NSP : 29,9 %</t>
+  </si>
+  <si>
+    <t>Le Pen vs Attal</t>
+  </si>
+  <si>
+    <t>NSP : 28,6 %</t>
+  </si>
+  <si>
+    <t>Union de la gauche hors LFI</t>
+  </si>
+  <si>
+    <t>PS candidat Glucksmann</t>
+  </si>
+  <si>
+    <t>RN : Le Pen ; PS : Glucksmann</t>
+  </si>
+  <si>
+    <t>NSP : 29,9 % !!</t>
+  </si>
+  <si>
+    <t>RN : Bardella ; PS : Glucksmann Correction manuelle pour intégrer MLP : RN -1,5, LR +0,75, Centre + 0,75</t>
+  </si>
+  <si>
+    <t>PS : Glucksmann</t>
+  </si>
+  <si>
+    <t>Marine Le Pen</t>
+  </si>
+  <si>
+    <t>Gabriel Attal</t>
+  </si>
+  <si>
+    <t>Jean-Luc Mélenchon</t>
+  </si>
+  <si>
+    <t>Attal + Glucksmann</t>
+  </si>
+  <si>
+    <t>Philippe + Hollande</t>
+  </si>
+  <si>
+    <t>Attal + Hollande</t>
+  </si>
+  <si>
+    <t>Mélenchon</t>
+  </si>
+  <si>
+    <t>De Villepin comptabilisé, 14 % d'abstention</t>
+  </si>
+  <si>
+    <t>De Villepin : 3,5</t>
+  </si>
+  <si>
+    <t>EELV : Ruffin+ Hollande+Philippe</t>
+  </si>
+  <si>
+    <t>De Villepin pas testé</t>
+  </si>
+  <si>
+    <t>Hollande+Philippe</t>
+  </si>
+  <si>
+    <t>De Villepin : 3</t>
+  </si>
+  <si>
+    <t>Abstention 29 %</t>
+  </si>
+  <si>
+    <t>Glucksman+Attal</t>
+  </si>
+  <si>
+    <t>Glucksman+Attal+philippe+Le Pen</t>
+  </si>
+  <si>
+    <t>Hollande+Attal</t>
+  </si>
+  <si>
+    <t>Philippe + Glucksmann union des gauches</t>
+  </si>
+  <si>
+    <t>Attal + Glucksmann union des gauches</t>
+  </si>
+  <si>
+    <t>Philippe + Hollande union des gauches</t>
+  </si>
+  <si>
+    <t>Le Maire candidat</t>
+  </si>
+  <si>
+    <t>Cluster17</t>
+  </si>
+  <si>
+    <t>De villepin 2,9 %, NDA 3,2</t>
+  </si>
+  <si>
+    <t>Villepin 3,9</t>
+  </si>
+  <si>
+    <t>Faure + Philippe</t>
+  </si>
+  <si>
+    <t>Faure + Attal</t>
+  </si>
+  <si>
+    <t>PS : Glucksmann ; Villepin candidat</t>
+  </si>
+  <si>
+    <t>Villepin 4</t>
+  </si>
+  <si>
+    <t>Attal + Philippe</t>
+  </si>
+  <si>
+    <t>Abstention 31 %</t>
+  </si>
+  <si>
+    <t>Philippe + glucksmann + Attal</t>
+  </si>
+  <si>
+    <t>Glucksman+Attal+philippe</t>
   </si>
 </sst>
 </file>
@@ -184,7 +319,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -211,6 +346,18 @@
         <fgColor rgb="FF3D3D3D"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -224,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -251,6 +398,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -684,7 +850,7 @@
       <c r="K3" s="4">
         <v>3</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="10" t="s">
         <v>16</v>
       </c>
     </row>
@@ -778,28 +944,28 @@
         <v>13</v>
       </c>
       <c r="E6" s="4">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G6" s="4">
         <v>3</v>
       </c>
       <c r="H6" s="4">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I6" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J6" s="4">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="K6" s="4">
         <v>6</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>14</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
@@ -819,30 +985,30 @@
         <v>13</v>
       </c>
       <c r="F7" s="2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G7" s="2">
         <v>4</v>
       </c>
       <c r="H7" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I7" s="2">
         <v>9</v>
       </c>
       <c r="J7" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K7" s="2">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B8" s="8">
         <v>46170</v>
@@ -863,230 +1029,590 @@
         <v>4</v>
       </c>
       <c r="H8" s="4">
+        <v>18.25</v>
+      </c>
+      <c r="I8" s="4">
+        <v>9.75</v>
+      </c>
+      <c r="J8" s="4">
+        <v>32.5</v>
+      </c>
+      <c r="K8" s="4">
+        <v>4</v>
+      </c>
+      <c r="L8" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="7">
+        <v>46184</v>
+      </c>
+      <c r="C9" s="2">
+        <v>901</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="2">
+        <v>13</v>
+      </c>
+      <c r="F9" s="2">
+        <v>13</v>
+      </c>
+      <c r="G9" s="2">
+        <v>5</v>
+      </c>
+      <c r="H9" s="2">
+        <v>19</v>
+      </c>
+      <c r="I9" s="2">
+        <v>8</v>
+      </c>
+      <c r="J9" s="2">
+        <v>33</v>
+      </c>
+      <c r="K9" s="2">
+        <v>3</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="8">
+        <v>46197</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1539</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="4">
+        <v>12</v>
+      </c>
+      <c r="F10" s="4">
+        <v>9</v>
+      </c>
+      <c r="G10" s="4">
+        <v>4</v>
+      </c>
+      <c r="H10" s="4">
+        <v>20</v>
+      </c>
+      <c r="I10" s="4">
+        <v>11</v>
+      </c>
+      <c r="J10" s="4">
+        <v>32</v>
+      </c>
+      <c r="K10" s="4">
+        <v>6</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="7">
+        <v>46211</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1075</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="2">
+        <v>15</v>
+      </c>
+      <c r="F11" s="2">
+        <v>9</v>
+      </c>
+      <c r="G11" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="H11" s="2">
+        <v>19</v>
+      </c>
+      <c r="I11" s="2">
+        <v>8</v>
+      </c>
+      <c r="J11" s="2">
+        <v>36</v>
+      </c>
+      <c r="K11" s="2">
+        <v>4</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="8">
+        <v>46211</v>
+      </c>
+      <c r="C12" s="4">
+        <v>1592</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="4">
+        <v>16</v>
+      </c>
+      <c r="F12" s="4">
+        <v>11</v>
+      </c>
+      <c r="G12" s="4">
+        <v>3</v>
+      </c>
+      <c r="H12" s="4">
+        <v>20</v>
+      </c>
+      <c r="I12" s="4">
+        <v>8</v>
+      </c>
+      <c r="J12" s="4">
+        <v>34</v>
+      </c>
+      <c r="K12" s="4">
+        <v>4</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="7">
+        <v>46212</v>
+      </c>
+      <c r="C13" s="2">
+        <v>963</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" s="2">
+        <v>15</v>
+      </c>
+      <c r="F13" s="2">
+        <v>9</v>
+      </c>
+      <c r="G13" s="2">
+        <v>4</v>
+      </c>
+      <c r="H13" s="2">
+        <v>22</v>
+      </c>
+      <c r="I13" s="2">
+        <v>9</v>
+      </c>
+      <c r="J13" s="2">
+        <v>34</v>
+      </c>
+      <c r="K13" s="2">
+        <v>4</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="8">
+        <v>46213</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1390</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="4">
+        <v>16</v>
+      </c>
+      <c r="F14" s="4">
+        <v>10.5</v>
+      </c>
+      <c r="G14" s="4">
+        <v>3.5</v>
+      </c>
+      <c r="H14" s="4">
+        <v>16.5</v>
+      </c>
+      <c r="I14" s="4">
+        <v>8</v>
+      </c>
+      <c r="J14" s="4">
+        <v>35</v>
+      </c>
+      <c r="K14" s="4">
+        <v>3</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="7">
+        <v>46253</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1764</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="2">
+        <v>17</v>
+      </c>
+      <c r="F15" s="2">
+        <v>10</v>
+      </c>
+      <c r="G15" s="2">
+        <v>3</v>
+      </c>
+      <c r="H15" s="2">
+        <v>17</v>
+      </c>
+      <c r="I15" s="2">
+        <v>7</v>
+      </c>
+      <c r="J15" s="2">
+        <v>35</v>
+      </c>
+      <c r="K15" s="2">
+        <v>4</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="4">
+        <v>17</v>
+      </c>
+      <c r="F16" s="4">
+        <v>12</v>
+      </c>
+      <c r="G16" s="4">
+        <v>3</v>
+      </c>
+      <c r="H16" s="4">
+        <v>18</v>
+      </c>
+      <c r="I16" s="4">
+        <v>8</v>
+      </c>
+      <c r="J16" s="4">
+        <v>33</v>
+      </c>
+      <c r="K16" s="4">
+        <v>3.5</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="7">
+        <v>46227</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1404</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="F17" s="2">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="G17" s="2">
+        <v>2.8</v>
+      </c>
+      <c r="H17" s="2">
+        <v>18.100000000000001</v>
+      </c>
+      <c r="I17" s="2">
+        <v>7.8</v>
+      </c>
+      <c r="J17" s="2">
+        <v>30.1</v>
+      </c>
+      <c r="K17" s="2">
+        <v>3.8</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="8">
+        <v>46267</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1500</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="4">
+        <v>15</v>
+      </c>
+      <c r="F18" s="4">
+        <v>12</v>
+      </c>
+      <c r="G18" s="4">
+        <v>4</v>
+      </c>
+      <c r="H18" s="4">
+        <v>19</v>
+      </c>
+      <c r="I18" s="4">
+        <v>7.5</v>
+      </c>
+      <c r="J18" s="4">
+        <v>34.5</v>
+      </c>
+      <c r="K18" s="4">
+        <v>3</v>
+      </c>
+      <c r="L18" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="7">
+        <v>46266</v>
+      </c>
+      <c r="C19" s="2">
+        <v>1628</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="2">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="F19" s="2">
+        <v>11.6</v>
+      </c>
+      <c r="G19" s="2">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="H19" s="2">
+        <v>18.2</v>
+      </c>
+      <c r="I19" s="2">
+        <v>7.5</v>
+      </c>
+      <c r="J19" s="2">
+        <v>30</v>
+      </c>
+      <c r="K19" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="8">
+        <v>46268</v>
+      </c>
+      <c r="C20" s="4">
+        <v>929</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" s="4">
+        <v>16</v>
+      </c>
+      <c r="F20" s="4">
+        <v>12</v>
+      </c>
+      <c r="G20" s="4">
+        <v>4</v>
+      </c>
+      <c r="H20" s="4">
+        <v>20</v>
+      </c>
+      <c r="I20" s="4">
+        <v>8</v>
+      </c>
+      <c r="J20" s="4">
+        <v>33</v>
+      </c>
+      <c r="K20" s="4">
+        <v>3</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="7">
+        <v>46274</v>
+      </c>
+      <c r="C21" s="2">
+        <v>948</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="2">
+        <v>15</v>
+      </c>
+      <c r="F21" s="2">
+        <v>10</v>
+      </c>
+      <c r="G21" s="2">
+        <v>3</v>
+      </c>
+      <c r="H21" s="2">
+        <v>19</v>
+      </c>
+      <c r="I21" s="2">
+        <v>10</v>
+      </c>
+      <c r="J21" s="2">
+        <v>34</v>
+      </c>
+      <c r="K21" s="2">
+        <v>4</v>
+      </c>
+      <c r="L21" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="8">
+        <v>46274</v>
+      </c>
+      <c r="C22" s="4">
+        <v>13060</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="4">
+        <v>15.5</v>
+      </c>
+      <c r="F22" s="4">
+        <v>12.5</v>
+      </c>
+      <c r="G22" s="4">
+        <v>4</v>
+      </c>
+      <c r="H22" s="4">
         <v>17.5</v>
       </c>
-      <c r="I8" s="4">
-        <v>9</v>
-      </c>
-      <c r="J8" s="4">
+      <c r="I22" s="4">
+        <v>8</v>
+      </c>
+      <c r="J22" s="4">
+        <v>33.5</v>
+      </c>
+      <c r="K22" s="4">
+        <v>4</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="7">
+        <v>46275</v>
+      </c>
+      <c r="C23" s="2">
+        <v>2052</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="2">
+        <v>17</v>
+      </c>
+      <c r="F23" s="2">
+        <v>10</v>
+      </c>
+      <c r="G23" s="2">
+        <v>3</v>
+      </c>
+      <c r="H23" s="2">
+        <v>17</v>
+      </c>
+      <c r="I23" s="2">
+        <v>7</v>
+      </c>
+      <c r="J23" s="2">
         <v>34</v>
       </c>
-      <c r="K8" s="4">
-        <v>4</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="3"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="5"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="3"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="5"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="3"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="5"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="3"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="5"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="3"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="5"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="3"/>
+      <c r="K23" s="2">
+        <v>5</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="4"/>
@@ -1236,16 +1762,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -1370,184 +1896,440 @@
       <c r="H6" s="5"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="7">
+        <v>46211</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1075</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="2">
+        <v>46</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="2">
+        <v>54</v>
+      </c>
       <c r="H7" s="3"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
+      <c r="A8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="8">
+        <v>46211</v>
+      </c>
+      <c r="C8" s="4">
+        <v>1075</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="4">
+        <v>45</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="4">
+        <v>55</v>
+      </c>
       <c r="H8" s="5"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="7">
+        <v>46211</v>
+      </c>
+      <c r="C9" s="2">
+        <v>1075</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="2">
+        <v>30</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="2">
+        <v>70</v>
+      </c>
       <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
+      <c r="A10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="8">
+        <v>46211</v>
+      </c>
+      <c r="C10" s="4">
+        <v>1592</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="4">
+        <v>33</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="4">
+        <v>67</v>
+      </c>
       <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="7">
+        <v>46211</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1592</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="2">
+        <v>45</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="2">
+        <v>55</v>
+      </c>
       <c r="H11" s="3"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+      <c r="A12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="8">
+        <v>46211</v>
+      </c>
+      <c r="C12" s="4">
+        <v>1592</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="4">
+        <v>49</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" s="4">
+        <v>51</v>
+      </c>
       <c r="H12" s="5"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="3"/>
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="7">
+        <v>46213</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1390</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="2">
+        <v>67.5</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
+      <c r="A14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="8">
+        <v>46213</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1390</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="4">
+        <v>46</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" s="4">
+        <v>54</v>
+      </c>
       <c r="H14" s="5"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="7">
+        <v>46213</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1390</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="2">
+        <v>48</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15" s="2">
+        <v>52</v>
+      </c>
       <c r="H15" s="3"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
+      <c r="A16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="4">
+        <v>48</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G16" s="4">
+        <v>52</v>
+      </c>
       <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="7">
+        <v>46259</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1598</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" s="2">
+        <v>46</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G17" s="2">
+        <v>54</v>
+      </c>
       <c r="H17" s="3"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
+      <c r="A18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="4">
+        <v>33</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" s="4">
+        <v>67</v>
+      </c>
       <c r="H18" s="5"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="A19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="7">
+        <v>46227</v>
+      </c>
+      <c r="C19" s="2">
+        <v>1404</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="2">
+        <v>48.2</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G19" s="2">
+        <v>51.8</v>
+      </c>
       <c r="H19" s="3"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="5"/>
+    <row r="20" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="12">
+        <v>46227</v>
+      </c>
+      <c r="C20" s="11">
+        <v>1404</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="11">
+        <v>39.200000000000003</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" s="11">
+        <v>60.8</v>
+      </c>
+      <c r="H20" s="13"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="A21" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" s="7">
+        <v>46227</v>
+      </c>
+      <c r="C21" s="2">
+        <v>1404</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="2">
+        <v>43.8</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G21" s="2">
+        <v>56.2</v>
+      </c>
       <c r="H21" s="3"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="A22" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="8">
+        <v>46268</v>
+      </c>
+      <c r="C22" s="4">
+        <v>929</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="4">
+        <v>45</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G22" s="4">
+        <v>55</v>
+      </c>
       <c r="H22" s="5"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+      <c r="A23" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="16">
+        <v>46268</v>
+      </c>
+      <c r="C23" s="15">
+        <v>929</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E23" s="2">
+        <v>48</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G23" s="2">
+        <v>52</v>
+      </c>
       <c r="H23" s="3"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="5"/>
+      <c r="A24" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="8">
+        <v>46268</v>
+      </c>
+      <c r="C24" s="4">
+        <v>929</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="4">
+        <v>34</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G24" s="4">
+        <v>66</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
@@ -1640,7 +2422,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1650,19 +2432,19 @@
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="8" max="9" width="9" customWidth="1"/>
+    <col min="10" max="10" width="7" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1685,22 +2467,25 @@
         <v>6</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1725,20 +2510,20 @@
       <c r="H3">
         <v>16</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>10</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>34</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>3</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1763,20 +2548,20 @@
       <c r="H4">
         <v>19</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>9</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>33</v>
       </c>
-      <c r="K4">
-        <v>4</v>
-      </c>
-      <c r="L4" t="s">
+      <c r="L4">
+        <v>4</v>
+      </c>
+      <c r="M4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1801,20 +2586,20 @@
       <c r="H5">
         <v>20</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>9</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>34</v>
       </c>
-      <c r="K5">
-        <v>4</v>
-      </c>
-      <c r="L5" t="s">
+      <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1839,22 +2624,22 @@
       <c r="H6">
         <v>16</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>11.5</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>32</v>
       </c>
-      <c r="K6">
-        <v>4</v>
-      </c>
-      <c r="L6" t="s">
+      <c r="L6">
+        <v>4</v>
+      </c>
+      <c r="M6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="9">
         <v>46170</v>
@@ -1863,7 +2648,7 @@
         <v>1500</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E7">
         <v>13</v>
@@ -1877,19 +2662,19 @@
       <c r="H7">
         <v>14.5</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>10</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>35</v>
       </c>
-      <c r="K7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B8" s="9">
         <v>46170</v>
@@ -1898,7 +2683,7 @@
         <v>1500</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E8">
         <v>13.5</v>
@@ -1912,19 +2697,19 @@
       <c r="H8">
         <v>19</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>9</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>35.5</v>
       </c>
-      <c r="K8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B9" s="9">
         <v>46170</v>
@@ -1933,7 +2718,7 @@
         <v>1500</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="E9">
         <v>13</v>
@@ -1947,18 +2732,18 @@
       <c r="H9">
         <v>14</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>8.5</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>31</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>4.5</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>17</v>
       </c>
       <c r="B10" s="9">
@@ -1968,7 +2753,7 @@
         <v>1744</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E10">
         <v>15</v>
@@ -1982,18 +2767,18 @@
       <c r="H10">
         <v>14</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>10</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>34</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" s="9">
@@ -2003,7 +2788,7 @@
         <v>1744</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E11">
         <v>14</v>
@@ -2017,18 +2802,18 @@
       <c r="H11">
         <v>19</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>10</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>31</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="9">
@@ -2038,7 +2823,7 @@
         <v>1744</v>
       </c>
       <c r="D12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E12">
         <v>15</v>
@@ -2052,14 +2837,1359 @@
       <c r="H12">
         <v>15</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>11</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>32</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="9">
+        <v>46184</v>
+      </c>
+      <c r="C13">
+        <v>901</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13">
+        <v>13</v>
+      </c>
+      <c r="F13">
+        <v>14</v>
+      </c>
+      <c r="G13">
+        <v>4</v>
+      </c>
+      <c r="H13">
+        <v>14</v>
+      </c>
+      <c r="J13">
+        <v>9</v>
+      </c>
+      <c r="K13">
+        <v>35</v>
+      </c>
+      <c r="L13">
+        <v>4</v>
+      </c>
+      <c r="M13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="9">
+        <v>46197</v>
+      </c>
+      <c r="C14">
+        <v>1539</v>
+      </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14">
+        <v>13</v>
+      </c>
+      <c r="F14">
+        <v>11</v>
+      </c>
+      <c r="G14">
+        <v>3.5</v>
+      </c>
+      <c r="H14">
+        <v>15</v>
+      </c>
+      <c r="J14">
+        <v>11</v>
+      </c>
+      <c r="K14">
+        <v>37</v>
+      </c>
+      <c r="L14">
+        <v>4.5</v>
+      </c>
+      <c r="M14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="9">
+        <v>46197</v>
+      </c>
+      <c r="C15">
+        <v>1539</v>
+      </c>
+      <c r="D15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15">
+        <v>12</v>
+      </c>
+      <c r="F15">
+        <v>9</v>
+      </c>
+      <c r="G15">
+        <v>4</v>
+      </c>
+      <c r="H15">
+        <v>20</v>
+      </c>
+      <c r="J15">
+        <v>11</v>
+      </c>
+      <c r="K15">
+        <v>32</v>
+      </c>
+      <c r="L15">
+        <v>6</v>
+      </c>
+      <c r="M15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="9">
+        <v>46197</v>
+      </c>
+      <c r="C16">
+        <v>1539</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16">
+        <v>13</v>
+      </c>
+      <c r="F16">
+        <v>11</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
+        <v>15</v>
+      </c>
+      <c r="J16">
+        <v>14</v>
+      </c>
+      <c r="K16">
+        <v>32</v>
+      </c>
+      <c r="L16">
+        <v>5</v>
+      </c>
+      <c r="M16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="9">
+        <v>46197</v>
+      </c>
+      <c r="C17">
+        <v>1539</v>
+      </c>
+      <c r="D17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17">
+        <v>14</v>
+      </c>
+      <c r="F17">
+        <v>11</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>20</v>
+      </c>
+      <c r="J17">
+        <v>11</v>
+      </c>
+      <c r="K17">
+        <v>36</v>
+      </c>
+      <c r="L17">
+        <v>4</v>
+      </c>
+      <c r="M17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="9">
+        <v>46211</v>
+      </c>
+      <c r="C18">
+        <v>1075</v>
+      </c>
+      <c r="D18" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18">
+        <v>15</v>
+      </c>
+      <c r="F18">
+        <v>12</v>
+      </c>
+      <c r="G18">
+        <v>4</v>
+      </c>
+      <c r="H18">
+        <v>15</v>
+      </c>
+      <c r="J18">
+        <v>10</v>
+      </c>
+      <c r="K18">
+        <v>36</v>
+      </c>
+      <c r="L18">
+        <v>3.5</v>
+      </c>
+      <c r="M18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="9">
+        <v>46211</v>
+      </c>
+      <c r="C19">
+        <v>1592</v>
+      </c>
+      <c r="D19" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19">
+        <v>16</v>
+      </c>
+      <c r="F19">
+        <v>11</v>
+      </c>
+      <c r="G19">
+        <v>3</v>
+      </c>
+      <c r="H19">
+        <v>16</v>
+      </c>
+      <c r="J19">
+        <v>9</v>
+      </c>
+      <c r="K19">
+        <v>36</v>
+      </c>
+      <c r="L19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="9">
+        <v>46211</v>
+      </c>
+      <c r="C20">
+        <v>1592</v>
+      </c>
+      <c r="D20" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20">
+        <v>16</v>
+      </c>
+      <c r="F20">
+        <v>8</v>
+      </c>
+      <c r="G20">
+        <v>4</v>
+      </c>
+      <c r="H20">
+        <v>20</v>
+      </c>
+      <c r="J20">
+        <v>8</v>
+      </c>
+      <c r="K20">
+        <v>35</v>
+      </c>
+      <c r="L20">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="9">
+        <v>46211</v>
+      </c>
+      <c r="C21">
+        <v>1592</v>
+      </c>
+      <c r="D21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21">
+        <v>16</v>
+      </c>
+      <c r="F21">
+        <v>8</v>
+      </c>
+      <c r="G21">
+        <v>5</v>
+      </c>
+      <c r="H21">
+        <v>16</v>
+      </c>
+      <c r="J21">
+        <v>8</v>
+      </c>
+      <c r="K21">
+        <v>36</v>
+      </c>
+      <c r="L21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="9">
+        <v>46212</v>
+      </c>
+      <c r="C22">
+        <v>963</v>
+      </c>
+      <c r="D22" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22">
+        <v>15</v>
+      </c>
+      <c r="F22">
+        <v>10</v>
+      </c>
+      <c r="G22">
+        <v>5</v>
+      </c>
+      <c r="H22">
+        <v>16</v>
+      </c>
+      <c r="J22">
+        <v>12</v>
+      </c>
+      <c r="K22">
+        <v>36</v>
+      </c>
+      <c r="L22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B23" s="9">
+        <v>46213</v>
+      </c>
+      <c r="C23">
+        <v>1390</v>
+      </c>
+      <c r="D23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23">
+        <v>14.5</v>
+      </c>
+      <c r="F23">
+        <v>11</v>
+      </c>
+      <c r="G23">
+        <v>3.5</v>
+      </c>
+      <c r="H23">
+        <v>13.5</v>
+      </c>
+      <c r="J23">
+        <v>11</v>
+      </c>
+      <c r="K23">
+        <v>34</v>
+      </c>
+      <c r="L23">
+        <v>3.5</v>
+      </c>
+      <c r="M23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="9">
+        <v>46213</v>
+      </c>
+      <c r="C24">
+        <v>1390</v>
+      </c>
+      <c r="D24" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24">
+        <v>14.5</v>
+      </c>
+      <c r="F24">
+        <v>9</v>
+      </c>
+      <c r="G24">
+        <v>6</v>
+      </c>
+      <c r="H24">
+        <v>19</v>
+      </c>
+      <c r="J24">
+        <v>9</v>
+      </c>
+      <c r="K24">
+        <v>35</v>
+      </c>
+      <c r="L24">
+        <v>2.5</v>
+      </c>
+      <c r="M24" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="9">
+        <v>46213</v>
+      </c>
+      <c r="C25">
+        <v>1390</v>
+      </c>
+      <c r="D25" t="s">
+        <v>68</v>
+      </c>
+      <c r="E25">
+        <v>15</v>
+      </c>
+      <c r="F25">
+        <v>8</v>
+      </c>
+      <c r="G25">
+        <v>4</v>
+      </c>
+      <c r="H25">
+        <v>18</v>
+      </c>
+      <c r="J25">
+        <v>8</v>
+      </c>
+      <c r="K25">
+        <v>34.5</v>
+      </c>
+      <c r="L25">
+        <v>3</v>
+      </c>
+      <c r="M25" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="7">
+        <v>46253</v>
+      </c>
+      <c r="C26" s="2">
+        <v>1764</v>
+      </c>
+      <c r="D26" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26">
+        <v>17</v>
+      </c>
+      <c r="F26">
+        <v>11</v>
+      </c>
+      <c r="G26">
+        <v>3</v>
+      </c>
+      <c r="H26">
+        <v>15</v>
+      </c>
+      <c r="J26">
+        <v>9</v>
+      </c>
+      <c r="K26">
+        <v>37</v>
+      </c>
+      <c r="L26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="7">
+        <v>46253</v>
+      </c>
+      <c r="C27" s="2">
+        <v>1764</v>
+      </c>
+      <c r="D27" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27">
+        <v>17</v>
+      </c>
+      <c r="F27">
+        <v>8</v>
+      </c>
+      <c r="G27">
+        <v>4</v>
+      </c>
+      <c r="H27">
+        <v>19</v>
+      </c>
+      <c r="J27">
+        <v>7</v>
+      </c>
+      <c r="K27">
+        <v>35</v>
+      </c>
+      <c r="L27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="7">
+        <v>46253</v>
+      </c>
+      <c r="C28" s="2">
+        <v>1764</v>
+      </c>
+      <c r="D28" t="s">
+        <v>73</v>
+      </c>
+      <c r="E28">
+        <v>17</v>
+      </c>
+      <c r="F28">
+        <v>8</v>
+      </c>
+      <c r="G28">
+        <v>4</v>
+      </c>
+      <c r="H28">
+        <v>14</v>
+      </c>
+      <c r="J28">
+        <v>9</v>
+      </c>
+      <c r="K28">
+        <v>38</v>
+      </c>
+      <c r="L28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C29" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D29" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29">
+        <v>17</v>
+      </c>
+      <c r="F29">
+        <v>15</v>
+      </c>
+      <c r="G29">
+        <v>3</v>
+      </c>
+      <c r="H29">
+        <v>14</v>
+      </c>
+      <c r="J29">
+        <v>9</v>
+      </c>
+      <c r="K29">
+        <v>34</v>
+      </c>
+      <c r="L29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C30" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D30" t="s">
+        <v>74</v>
+      </c>
+      <c r="E30">
+        <v>18</v>
+      </c>
+      <c r="F30">
+        <v>15</v>
+      </c>
+      <c r="H30">
+        <v>19</v>
+      </c>
+      <c r="J30">
+        <v>8</v>
+      </c>
+      <c r="K30">
+        <v>33</v>
+      </c>
+      <c r="L30">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C31" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D31" t="s">
+        <v>75</v>
+      </c>
+      <c r="E31">
+        <v>18.5</v>
+      </c>
+      <c r="F31">
+        <v>17</v>
+      </c>
+      <c r="H31">
+        <v>15</v>
+      </c>
+      <c r="J31">
+        <v>9</v>
+      </c>
+      <c r="K31">
+        <v>34</v>
+      </c>
+      <c r="L31">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C32" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D32" t="s">
+        <v>76</v>
+      </c>
+      <c r="E32">
+        <v>19</v>
+      </c>
+      <c r="F32">
+        <v>12</v>
+      </c>
+      <c r="H32">
+        <v>21</v>
+      </c>
+      <c r="J32">
+        <v>8</v>
+      </c>
+      <c r="K32">
+        <v>34</v>
+      </c>
+      <c r="L32">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="8">
+        <v>46259</v>
+      </c>
+      <c r="C33" s="4">
+        <v>1598</v>
+      </c>
+      <c r="D33" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33">
+        <v>17</v>
+      </c>
+      <c r="F33">
+        <v>18</v>
+      </c>
+      <c r="G33">
+        <v>3</v>
+      </c>
+      <c r="H33">
+        <v>6</v>
+      </c>
+      <c r="J33">
+        <v>12</v>
+      </c>
+      <c r="K33">
+        <v>35</v>
+      </c>
+      <c r="L33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="7">
+        <v>46227</v>
+      </c>
+      <c r="C34" s="2">
+        <v>1404</v>
+      </c>
+      <c r="D34" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34">
+        <v>18.3</v>
+      </c>
+      <c r="F34">
+        <v>10.3</v>
+      </c>
+      <c r="G34">
+        <v>3.1</v>
+      </c>
+      <c r="H34">
+        <v>13.8</v>
+      </c>
+      <c r="J34">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="K34">
+        <v>29.9</v>
+      </c>
+      <c r="L34">
+        <v>4.2</v>
+      </c>
+      <c r="M34" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A35" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" s="8">
+        <v>46267</v>
+      </c>
+      <c r="C35" s="4">
+        <v>1500</v>
+      </c>
+      <c r="D35" t="s">
+        <v>60</v>
+      </c>
+      <c r="E35">
+        <v>15</v>
+      </c>
+      <c r="F35">
+        <v>14</v>
+      </c>
+      <c r="G35">
+        <v>4</v>
+      </c>
+      <c r="H35">
+        <v>14</v>
+      </c>
+      <c r="J35">
+        <v>9.5</v>
+      </c>
+      <c r="K35">
+        <v>35</v>
+      </c>
+      <c r="L35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" s="8">
+        <v>46267</v>
+      </c>
+      <c r="C36" s="4">
+        <v>1500</v>
+      </c>
+      <c r="D36" t="s">
+        <v>81</v>
+      </c>
+      <c r="E36">
+        <v>16.5</v>
+      </c>
+      <c r="F36">
+        <v>4.5</v>
+      </c>
+      <c r="G36">
+        <v>5</v>
+      </c>
+      <c r="H36">
+        <v>22.5</v>
+      </c>
+      <c r="J36">
+        <v>7.5</v>
+      </c>
+      <c r="K36">
+        <v>34.5</v>
+      </c>
+      <c r="L36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="8">
+        <v>46267</v>
+      </c>
+      <c r="C37" s="4">
+        <v>1500</v>
+      </c>
+      <c r="D37" t="s">
+        <v>82</v>
+      </c>
+      <c r="E37">
+        <v>17</v>
+      </c>
+      <c r="F37">
+        <v>5.5</v>
+      </c>
+      <c r="G37">
+        <v>5.5</v>
+      </c>
+      <c r="H37">
+        <v>15.5</v>
+      </c>
+      <c r="J37">
+        <v>10</v>
+      </c>
+      <c r="K37">
+        <v>36</v>
+      </c>
+      <c r="L37">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="8">
+        <v>46267</v>
+      </c>
+      <c r="C38" s="4">
+        <v>1500</v>
+      </c>
+      <c r="D38" t="s">
+        <v>87</v>
+      </c>
+      <c r="E38">
+        <v>15</v>
+      </c>
+      <c r="F38">
+        <v>11.5</v>
+      </c>
+      <c r="G38">
+        <v>3.5</v>
+      </c>
+      <c r="H38">
+        <v>14.5</v>
+      </c>
+      <c r="I38">
+        <v>7.5</v>
+      </c>
+      <c r="J38">
+        <v>6</v>
+      </c>
+      <c r="K38">
+        <v>34</v>
+      </c>
+      <c r="L38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="7">
+        <v>46266</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1628</v>
+      </c>
+      <c r="D39" t="s">
+        <v>60</v>
+      </c>
+      <c r="E39">
+        <v>18.2</v>
+      </c>
+      <c r="F39">
+        <v>11.5</v>
+      </c>
+      <c r="G39">
+        <v>2.5</v>
+      </c>
+      <c r="H39">
+        <v>13.5</v>
+      </c>
+      <c r="J39">
+        <v>8.9</v>
+      </c>
+      <c r="K39">
+        <v>31.6</v>
+      </c>
+      <c r="L39">
+        <v>4</v>
+      </c>
+      <c r="M39" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="8">
+        <v>46268</v>
+      </c>
+      <c r="C40" s="4">
+        <v>929</v>
+      </c>
+      <c r="D40" t="s">
+        <v>60</v>
+      </c>
+      <c r="E40">
+        <v>17</v>
+      </c>
+      <c r="F40">
+        <v>13</v>
+      </c>
+      <c r="G40">
+        <v>4</v>
+      </c>
+      <c r="I40">
+        <v>13</v>
+      </c>
+      <c r="J40">
+        <v>11</v>
+      </c>
+      <c r="K40">
+        <v>35</v>
+      </c>
+      <c r="L40">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="8">
+        <v>46268</v>
+      </c>
+      <c r="C41" s="4">
+        <v>929</v>
+      </c>
+      <c r="D41" t="s">
+        <v>85</v>
+      </c>
+      <c r="E41">
+        <v>17</v>
+      </c>
+      <c r="F41">
+        <v>11</v>
+      </c>
+      <c r="G41">
+        <v>3</v>
+      </c>
+      <c r="H41">
+        <v>15</v>
+      </c>
+      <c r="I41">
+        <v>7</v>
+      </c>
+      <c r="J41">
+        <v>7</v>
+      </c>
+      <c r="K41">
+        <v>34</v>
+      </c>
+      <c r="L41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" s="7">
+        <v>46274</v>
+      </c>
+      <c r="C42" s="2">
+        <v>948</v>
+      </c>
+      <c r="D42" t="s">
+        <v>44</v>
+      </c>
+      <c r="E42">
+        <v>15</v>
+      </c>
+      <c r="F42">
+        <v>12</v>
+      </c>
+      <c r="G42">
+        <v>4</v>
+      </c>
+      <c r="I42">
+        <v>14</v>
+      </c>
+      <c r="J42">
+        <v>12</v>
+      </c>
+      <c r="K42">
+        <v>34</v>
+      </c>
+      <c r="L42">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="7">
+        <v>46274</v>
+      </c>
+      <c r="C43" s="2">
+        <v>948</v>
+      </c>
+      <c r="D43" t="s">
+        <v>85</v>
+      </c>
+      <c r="E43">
+        <v>15</v>
+      </c>
+      <c r="F43">
+        <v>9</v>
+      </c>
+      <c r="G43">
+        <v>3</v>
+      </c>
+      <c r="H43">
+        <v>15</v>
+      </c>
+      <c r="I43">
+        <v>8</v>
+      </c>
+      <c r="J43">
+        <v>8</v>
+      </c>
+      <c r="K43">
+        <v>34</v>
+      </c>
+      <c r="L43">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A44" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B44" s="8">
+        <v>46274</v>
+      </c>
+      <c r="C44" s="4">
+        <v>13060</v>
+      </c>
+      <c r="D44" t="s">
+        <v>85</v>
+      </c>
+      <c r="E44">
+        <v>15.5</v>
+      </c>
+      <c r="F44">
+        <v>11.5</v>
+      </c>
+      <c r="G44">
+        <v>4</v>
+      </c>
+      <c r="H44">
+        <v>14</v>
+      </c>
+      <c r="I44">
+        <v>6</v>
+      </c>
+      <c r="J44">
+        <v>7</v>
+      </c>
+      <c r="K44">
+        <v>33</v>
+      </c>
+      <c r="L44">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A45" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" s="8">
+        <v>46274</v>
+      </c>
+      <c r="C45" s="4">
+        <v>13060</v>
+      </c>
+      <c r="D45" t="s">
+        <v>44</v>
+      </c>
+      <c r="E45">
+        <v>15.5</v>
+      </c>
+      <c r="F45">
+        <v>13.5</v>
+      </c>
+      <c r="G45">
+        <v>4.5</v>
+      </c>
+      <c r="I45">
+        <v>13</v>
+      </c>
+      <c r="J45">
+        <v>10</v>
+      </c>
+      <c r="K45">
+        <v>34</v>
+      </c>
+      <c r="L45">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B46" s="7">
+        <v>46275</v>
+      </c>
+      <c r="C46" s="2">
+        <v>2052</v>
+      </c>
+      <c r="D46" t="s">
+        <v>88</v>
+      </c>
+      <c r="E46">
+        <v>16</v>
+      </c>
+      <c r="F46">
+        <v>9</v>
+      </c>
+      <c r="G46">
+        <v>3</v>
+      </c>
+      <c r="H46">
+        <v>14</v>
+      </c>
+      <c r="I46">
+        <v>8</v>
+      </c>
+      <c r="J46">
+        <v>7</v>
+      </c>
+      <c r="K46">
+        <v>33</v>
+      </c>
+      <c r="L46">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B47" s="7">
+        <v>46275</v>
+      </c>
+      <c r="C47" s="2">
+        <v>2052</v>
+      </c>
+      <c r="D47" t="s">
+        <v>60</v>
+      </c>
+      <c r="E47">
+        <v>17</v>
+      </c>
+      <c r="F47">
+        <v>12</v>
+      </c>
+      <c r="G47">
+        <v>3</v>
+      </c>
+      <c r="I47">
+        <v>14</v>
+      </c>
+      <c r="J47">
+        <v>9</v>
+      </c>
+      <c r="K47">
+        <v>35</v>
+      </c>
+      <c r="L47">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B48" s="7">
+        <v>46275</v>
+      </c>
+      <c r="C48" s="2">
+        <v>2052</v>
+      </c>
+      <c r="D48" t="s">
+        <v>68</v>
+      </c>
+      <c r="E48">
+        <v>17</v>
+      </c>
+      <c r="F48">
+        <v>7</v>
+      </c>
+      <c r="G48">
+        <v>4</v>
+      </c>
+      <c r="H48">
+        <v>19</v>
+      </c>
+      <c r="J48">
+        <v>9</v>
+      </c>
+      <c r="K48">
+        <v>33</v>
+      </c>
+      <c r="L48">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="7">
+        <v>46275</v>
+      </c>
+      <c r="C49" s="2">
+        <v>2052</v>
+      </c>
+      <c r="D49" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49">
+        <v>17</v>
+      </c>
+      <c r="F49">
+        <v>7</v>
+      </c>
+      <c r="G49">
+        <v>4</v>
+      </c>
+      <c r="I49">
+        <v>15</v>
+      </c>
+      <c r="J49">
+        <v>10</v>
+      </c>
+      <c r="K49">
+        <v>36</v>
+      </c>
+      <c r="L49">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B50" s="7">
+        <v>46275</v>
+      </c>
+      <c r="C50" s="2">
+        <v>2052</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Plafonner l'échantillon à 3000 dans la pondération ; conserver la série sans plafond
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sondages_2027.xlsx
+++ b/sondages_2027.xlsx
@@ -1,28 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Projets/agregateur-sondages-2027/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F8FB31-A090-B445-ABDD-387BF9632EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17467214-A137-4B46-9DD7-9A2D4DF41B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="500" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T1 — intentions de vote" sheetId="1" r:id="rId1"/>
     <sheet name="T2 — hypothèses (référence)" sheetId="2" r:id="rId2"/>
     <sheet name="T1 — scénarios alternatifs" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="103">
   <si>
     <t>Institut</t>
   </si>
@@ -238,9 +238,6 @@
     <t>Abstention 29 %</t>
   </si>
   <si>
-    <t>Glucksman+Attal</t>
-  </si>
-  <si>
     <t>Glucksman+Attal+philippe+Le Pen</t>
   </si>
   <si>
@@ -290,6 +287,51 @@
   </si>
   <si>
     <t>Glucksman+Attal+philippe</t>
+  </si>
+  <si>
+    <t>Zemmour pas testé ; Lisnard 5,2 %</t>
+  </si>
+  <si>
+    <t>Philippe + Royal</t>
+  </si>
+  <si>
+    <t>Attal + Faure</t>
+  </si>
+  <si>
+    <t>Philippe + Faure</t>
+  </si>
+  <si>
+    <t>GLUCKSMANN OFFICIELEMENT CANDIDAT PS</t>
+  </si>
+  <si>
+    <t>Glucksmann</t>
+  </si>
+  <si>
+    <t>Lisnard 4</t>
+  </si>
+  <si>
+    <t>Philippe 13 ??? Sondage alternatif Lisnard 4 / retailleau 5</t>
+  </si>
+  <si>
+    <t>Lisnard 5,5</t>
+  </si>
+  <si>
+    <t>YouGov</t>
+  </si>
+  <si>
+    <t>Lisnard 7</t>
+  </si>
+  <si>
+    <t>Pas de candidat LR</t>
+  </si>
+  <si>
+    <t>Pas de centriste</t>
+  </si>
+  <si>
+    <t>Glucksmann union gauche</t>
+  </si>
+  <si>
+    <t>Philippe + Lisnard</t>
   </si>
 </sst>
 </file>
@@ -371,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -416,6 +458,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -723,7 +768,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -737,7 +782,7 @@
     <col min="9" max="9" width="7" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="12" max="12" width="81" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -1350,7 +1395,7 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17" s="7">
         <v>46227</v>
@@ -1383,7 +1428,7 @@
         <v>3.8</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
@@ -1426,7 +1471,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" s="7">
         <v>46266</v>
@@ -1459,7 +1504,7 @@
         <v>3.5</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
@@ -1615,130 +1660,1086 @@
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="5"/>
+      <c r="A24" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="8">
+        <v>46281</v>
+      </c>
+      <c r="C24" s="4">
+        <v>1943</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="4">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="F24" s="4">
+        <v>11.8</v>
+      </c>
+      <c r="G24" s="4">
+        <v>2.6</v>
+      </c>
+      <c r="H24" s="4">
+        <v>18.8</v>
+      </c>
+      <c r="I24" s="4">
+        <v>7.6</v>
+      </c>
+      <c r="J24" s="4">
+        <v>30.8</v>
+      </c>
+      <c r="K24" s="4">
+        <v>3.5</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="3"/>
+      <c r="A25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="7">
+        <v>46289</v>
+      </c>
+      <c r="C25" s="2">
+        <v>1974</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="2">
+        <v>18</v>
+      </c>
+      <c r="F25" s="2">
+        <v>10</v>
+      </c>
+      <c r="G25" s="2">
+        <v>3</v>
+      </c>
+      <c r="H25" s="2">
+        <v>16</v>
+      </c>
+      <c r="I25" s="2">
+        <v>8</v>
+      </c>
+      <c r="J25" s="2">
+        <v>35</v>
+      </c>
+      <c r="K25" s="2">
+        <v>5</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="5"/>
+      <c r="A26" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" s="8">
+        <v>46275</v>
+      </c>
+      <c r="C26" s="4">
+        <v>935</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" s="4">
+        <v>17</v>
+      </c>
+      <c r="F26" s="4">
+        <v>9</v>
+      </c>
+      <c r="G26" s="4">
+        <v>3</v>
+      </c>
+      <c r="H26" s="4">
+        <v>15</v>
+      </c>
+      <c r="I26" s="4">
+        <v>7</v>
+      </c>
+      <c r="J26" s="4">
+        <v>34</v>
+      </c>
+      <c r="K26" s="4">
+        <v>2</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-      <c r="J27" s="2"/>
-      <c r="K27" s="2"/>
-      <c r="L27" s="3"/>
+      <c r="A27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="7">
+        <v>46294</v>
+      </c>
+      <c r="C27" s="2">
+        <v>1527</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="2">
+        <v>16</v>
+      </c>
+      <c r="F27" s="2">
+        <v>11</v>
+      </c>
+      <c r="G27" s="2">
+        <v>3</v>
+      </c>
+      <c r="H27" s="2">
+        <v>21</v>
+      </c>
+      <c r="I27" s="2">
+        <v>8</v>
+      </c>
+      <c r="J27" s="2">
+        <v>33</v>
+      </c>
+      <c r="K27" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="L27" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="5"/>
+      <c r="A28" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="8">
+        <v>46303</v>
+      </c>
+      <c r="C28" s="4">
+        <v>2004</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" s="4">
+        <v>18</v>
+      </c>
+      <c r="F28" s="4">
+        <v>10</v>
+      </c>
+      <c r="G28" s="4">
+        <v>3</v>
+      </c>
+      <c r="H28" s="4">
+        <v>17</v>
+      </c>
+      <c r="I28" s="4">
+        <v>7</v>
+      </c>
+      <c r="J28" s="4">
+        <v>36</v>
+      </c>
+      <c r="K28" s="4">
+        <v>4</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="3"/>
+      <c r="A29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="7">
+        <v>46302</v>
+      </c>
+      <c r="C29" s="2">
+        <v>7599</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="2">
+        <v>18</v>
+      </c>
+      <c r="F29" s="2">
+        <v>9.5</v>
+      </c>
+      <c r="G29" s="2">
+        <v>3</v>
+      </c>
+      <c r="H29" s="2">
+        <v>17</v>
+      </c>
+      <c r="I29" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="J29" s="2">
+        <v>37</v>
+      </c>
+      <c r="K29" s="2">
+        <v>4.5</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="5"/>
+      <c r="A30" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="8">
+        <v>46309</v>
+      </c>
+      <c r="C30" s="4">
+        <v>1390</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" s="4">
+        <v>16</v>
+      </c>
+      <c r="F30" s="4">
+        <v>13.5</v>
+      </c>
+      <c r="G30" s="4">
+        <v>2.5</v>
+      </c>
+      <c r="H30" s="4">
+        <v>18</v>
+      </c>
+      <c r="I30" s="4">
+        <v>6.5</v>
+      </c>
+      <c r="J30" s="4">
+        <v>35</v>
+      </c>
+      <c r="K30" s="4">
+        <v>3</v>
+      </c>
+      <c r="L30" s="5" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
+      <c r="A31" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="7">
+        <v>46309</v>
+      </c>
+      <c r="C31" s="2">
+        <v>978</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="2">
+        <v>15</v>
+      </c>
+      <c r="F31" s="2">
+        <v>15</v>
+      </c>
+      <c r="G31" s="2">
+        <v>3</v>
+      </c>
+      <c r="H31" s="2">
+        <v>15</v>
+      </c>
+      <c r="I31" s="2">
+        <v>8</v>
+      </c>
+      <c r="J31" s="2">
+        <v>35</v>
+      </c>
+      <c r="K31" s="2">
+        <v>4</v>
+      </c>
       <c r="L31" s="3"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="5"/>
+      <c r="A32" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B32" s="8">
+        <v>46310</v>
+      </c>
+      <c r="C32" s="4">
+        <v>1094</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" s="4">
+        <v>15</v>
+      </c>
+      <c r="F32" s="4">
+        <v>13</v>
+      </c>
+      <c r="G32" s="4">
+        <v>6</v>
+      </c>
+      <c r="H32" s="4">
+        <v>13</v>
+      </c>
+      <c r="I32" s="4">
+        <v>7</v>
+      </c>
+      <c r="J32" s="4">
+        <v>36</v>
+      </c>
+      <c r="K32" s="4">
+        <v>3</v>
+      </c>
+      <c r="L32" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B33" s="7">
+        <v>46311</v>
+      </c>
+      <c r="C33" s="2">
+        <v>1701</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="F33" s="2">
+        <v>15</v>
+      </c>
+      <c r="G33" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="H33" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="I33" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="J33" s="2">
+        <v>31.5</v>
+      </c>
+      <c r="K33" s="2">
+        <v>3</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B34" s="8">
+        <v>46310</v>
+      </c>
+      <c r="C34" s="4">
+        <v>1187</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="4">
+        <v>18</v>
+      </c>
+      <c r="F34" s="4">
+        <v>11</v>
+      </c>
+      <c r="G34" s="4">
+        <v>2</v>
+      </c>
+      <c r="H34" s="4">
+        <v>17</v>
+      </c>
+      <c r="I34" s="4">
+        <v>7</v>
+      </c>
+      <c r="J34" s="4">
+        <v>31</v>
+      </c>
+      <c r="K34" s="4">
+        <v>3</v>
+      </c>
+      <c r="L34" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35" s="7">
+        <v>46314</v>
+      </c>
+      <c r="C35" s="2">
+        <v>1928</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" s="2">
+        <v>16.5</v>
+      </c>
+      <c r="F35" s="2">
+        <v>14</v>
+      </c>
+      <c r="G35" s="2">
+        <v>3</v>
+      </c>
+      <c r="H35" s="2">
+        <v>15</v>
+      </c>
+      <c r="I35" s="2">
+        <v>7.5</v>
+      </c>
+      <c r="J35" s="2">
+        <v>36</v>
+      </c>
+      <c r="K35" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="L35" s="3"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A36" s="4"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="5"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A37" s="2"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="3"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A38" s="4"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="5"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A39" s="2"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="3"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A40" s="4"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="5"/>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A41" s="2"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="3"/>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A42" s="4"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="5"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A43" s="2"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="3"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A44" s="4"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+      <c r="J44" s="4"/>
+      <c r="K44" s="4"/>
+      <c r="L44" s="5"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A45" s="2"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+      <c r="L45" s="3"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A46" s="4"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="5"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A47" s="2"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+      <c r="L47" s="3"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A48" s="4"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="4"/>
+      <c r="J48" s="4"/>
+      <c r="K48" s="4"/>
+      <c r="L48" s="5"/>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A49" s="2"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
+      <c r="K49" s="2"/>
+      <c r="L49" s="3"/>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A50" s="4"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="5"/>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A51" s="2"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
+      <c r="L51" s="3"/>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A52" s="4"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+      <c r="L52" s="5"/>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A53" s="2"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+      <c r="L53" s="3"/>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A54" s="4"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="5"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A55" s="2"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
+      <c r="L55" s="3"/>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A56" s="4"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+      <c r="I56" s="4"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="5"/>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A57" s="2"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
+      <c r="L57" s="3"/>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A58" s="4"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="5"/>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A59" s="2"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
+      <c r="L59" s="3"/>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A60" s="4"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
+      <c r="K60" s="4"/>
+      <c r="L60" s="5"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A61" s="2"/>
+      <c r="B61" s="7"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+      <c r="L61" s="3"/>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A62" s="4"/>
+      <c r="B62" s="8"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+      <c r="L62" s="5"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A63" s="2"/>
+      <c r="B63" s="7"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+      <c r="I63" s="2"/>
+      <c r="J63" s="2"/>
+      <c r="K63" s="2"/>
+      <c r="L63" s="3"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A64" s="4"/>
+      <c r="B64" s="8"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+      <c r="L64" s="5"/>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A65" s="2"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+      <c r="G65" s="2"/>
+      <c r="H65" s="2"/>
+      <c r="I65" s="2"/>
+      <c r="J65" s="2"/>
+      <c r="K65" s="2"/>
+      <c r="L65" s="3"/>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A66" s="4"/>
+      <c r="B66" s="8"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+      <c r="G66" s="4"/>
+      <c r="H66" s="4"/>
+      <c r="I66" s="4"/>
+      <c r="J66" s="4"/>
+      <c r="K66" s="4"/>
+      <c r="L66" s="5"/>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A67" s="2"/>
+      <c r="B67" s="7"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
+      <c r="F67" s="2"/>
+      <c r="G67" s="2"/>
+      <c r="H67" s="2"/>
+      <c r="I67" s="2"/>
+      <c r="J67" s="2"/>
+      <c r="K67" s="2"/>
+      <c r="L67" s="3"/>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A68" s="4"/>
+      <c r="B68" s="8"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
+      <c r="G68" s="4"/>
+      <c r="H68" s="4"/>
+      <c r="I68" s="4"/>
+      <c r="J68" s="4"/>
+      <c r="K68" s="4"/>
+      <c r="L68" s="5"/>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A69" s="2"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
+      <c r="F69" s="2"/>
+      <c r="G69" s="2"/>
+      <c r="H69" s="2"/>
+      <c r="I69" s="2"/>
+      <c r="J69" s="2"/>
+      <c r="K69" s="2"/>
+      <c r="L69" s="3"/>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A70" s="4"/>
+      <c r="B70" s="8"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+      <c r="H70" s="4"/>
+      <c r="I70" s="4"/>
+      <c r="J70" s="4"/>
+      <c r="K70" s="4"/>
+      <c r="L70" s="5"/>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A71" s="2"/>
+      <c r="B71" s="7"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
+      <c r="H71" s="2"/>
+      <c r="I71" s="2"/>
+      <c r="J71" s="2"/>
+      <c r="K71" s="2"/>
+      <c r="L71" s="3"/>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A72" s="4"/>
+      <c r="B72" s="8"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="4"/>
+      <c r="I72" s="4"/>
+      <c r="J72" s="4"/>
+      <c r="K72" s="4"/>
+      <c r="L72" s="5"/>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A73" s="2"/>
+      <c r="B73" s="7"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="2"/>
+      <c r="E73" s="2"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
+      <c r="H73" s="2"/>
+      <c r="I73" s="2"/>
+      <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
+      <c r="L73" s="3"/>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A74" s="4"/>
+      <c r="B74" s="8"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4"/>
+      <c r="F74" s="4"/>
+      <c r="G74" s="4"/>
+      <c r="H74" s="4"/>
+      <c r="I74" s="4"/>
+      <c r="J74" s="4"/>
+      <c r="K74" s="4"/>
+      <c r="L74" s="5"/>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A75" s="2"/>
+      <c r="B75" s="7"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="E75" s="2"/>
+      <c r="F75" s="2"/>
+      <c r="G75" s="2"/>
+      <c r="H75" s="2"/>
+      <c r="I75" s="2"/>
+      <c r="J75" s="2"/>
+      <c r="K75" s="2"/>
+      <c r="L75" s="3"/>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A76" s="4"/>
+      <c r="B76" s="8"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4"/>
+      <c r="E76" s="4"/>
+      <c r="F76" s="4"/>
+      <c r="G76" s="4"/>
+      <c r="H76" s="4"/>
+      <c r="I76" s="4"/>
+      <c r="J76" s="4"/>
+      <c r="K76" s="4"/>
+      <c r="L76" s="5"/>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A77" s="2"/>
+      <c r="B77" s="7"/>
+      <c r="C77" s="2"/>
+      <c r="D77" s="2"/>
+      <c r="E77" s="2"/>
+      <c r="F77" s="2"/>
+      <c r="G77" s="2"/>
+      <c r="H77" s="2"/>
+      <c r="I77" s="2"/>
+      <c r="J77" s="2"/>
+      <c r="K77" s="2"/>
+      <c r="L77" s="3"/>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A78" s="4"/>
+      <c r="B78" s="8"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
+      <c r="F78" s="4"/>
+      <c r="G78" s="4"/>
+      <c r="H78" s="4"/>
+      <c r="I78" s="4"/>
+      <c r="J78" s="4"/>
+      <c r="K78" s="4"/>
+      <c r="L78" s="5"/>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A79" s="2"/>
+      <c r="B79" s="7"/>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2"/>
+      <c r="E79" s="2"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
+      <c r="H79" s="2"/>
+      <c r="I79" s="2"/>
+      <c r="J79" s="2"/>
+      <c r="K79" s="2"/>
+      <c r="L79" s="3"/>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A80" s="4"/>
+      <c r="B80" s="8"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="4"/>
+      <c r="F80" s="4"/>
+      <c r="G80" s="4"/>
+      <c r="H80" s="4"/>
+      <c r="I80" s="4"/>
+      <c r="J80" s="4"/>
+      <c r="K80" s="4"/>
+      <c r="L80" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1748,7 +2749,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1762,16 +2763,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2187,7 +3188,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B19" s="7">
         <v>46227</v>
@@ -2211,7 +3212,7 @@
     </row>
     <row r="20" spans="1:8" s="14" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B20" s="12">
         <v>46227</v>
@@ -2235,7 +3236,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B21" s="7">
         <v>46227</v>
@@ -2328,88 +3329,756 @@
         <v>66</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
+      <c r="A25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="7">
+        <v>46289</v>
+      </c>
+      <c r="C25" s="2">
+        <v>1974</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E25" s="2">
+        <v>31</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G25" s="2">
+        <v>69</v>
+      </c>
       <c r="H25" s="3"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
+      <c r="A26" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="8">
+        <v>46289</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1974</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" s="4">
+        <v>43</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G26" s="4">
+        <v>57</v>
+      </c>
       <c r="H26" s="5"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="A27" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="7">
+        <v>46275</v>
+      </c>
+      <c r="C27" s="2">
+        <v>935</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" s="2">
+        <v>33</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G27" s="2">
+        <v>67</v>
+      </c>
       <c r="H27" s="3"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="A28" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B28" s="8">
+        <v>46275</v>
+      </c>
+      <c r="C28" s="4">
+        <v>935</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E28" s="4">
+        <v>45</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G28" s="4">
+        <v>55</v>
+      </c>
       <c r="H28" s="5"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
+      <c r="A29" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29" s="16">
+        <v>46303</v>
+      </c>
+      <c r="C29" s="15">
+        <v>2004</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="2">
+        <v>44</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G29" s="2">
+        <v>56</v>
+      </c>
       <c r="H29" s="3"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
+      <c r="A30" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="8">
+        <v>46303</v>
+      </c>
+      <c r="C30" s="4">
+        <v>2004</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E30" s="4">
+        <v>33</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G30" s="4">
+        <v>67</v>
+      </c>
       <c r="H30" s="5"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
+      <c r="A31" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="7">
+        <v>46302</v>
+      </c>
+      <c r="C31" s="2">
+        <v>7374</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="2">
+        <v>47</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G31" s="2">
+        <v>53</v>
+      </c>
       <c r="H31" s="3"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
+      <c r="A32" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" s="8">
+        <v>46302</v>
+      </c>
+      <c r="C32" s="4">
+        <v>6634</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E32" s="4">
+        <v>32</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G32" s="4">
+        <v>68</v>
+      </c>
       <c r="H32" s="5"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="7">
+        <v>46309</v>
+      </c>
+      <c r="C33" s="2">
+        <v>978</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E33" s="2">
+        <v>32</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G33" s="2">
+        <v>68</v>
+      </c>
+      <c r="H33" s="3"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="8">
+        <v>46309</v>
+      </c>
+      <c r="C34" s="4">
+        <v>978</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="4">
+        <v>44</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G34" s="4">
+        <v>56</v>
+      </c>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B35" s="7">
+        <v>46309</v>
+      </c>
+      <c r="C35" s="2">
+        <v>978</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E35" s="2">
+        <v>44</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G35" s="2">
+        <v>56</v>
+      </c>
+      <c r="H35" s="3"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B36" s="8">
+        <v>46311</v>
+      </c>
+      <c r="C36" s="4">
+        <v>1701</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E36" s="4">
+        <v>31</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G36" s="4">
+        <v>69</v>
+      </c>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" s="7">
+        <v>46311</v>
+      </c>
+      <c r="C37" s="2">
+        <v>1701</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E37" s="2">
+        <v>46.5</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G37" s="2">
+        <v>53.5</v>
+      </c>
+      <c r="H37" s="3"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B38" s="8">
+        <v>46311</v>
+      </c>
+      <c r="C38" s="4">
+        <v>1701</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" s="4">
+        <v>47.5</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G38" s="4">
+        <v>52.5</v>
+      </c>
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" s="7">
+        <v>46314</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1928</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E39" s="2">
+        <v>44</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G39" s="2">
+        <v>56</v>
+      </c>
+      <c r="H39" s="3"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="8">
+        <v>46314</v>
+      </c>
+      <c r="C40" s="4">
+        <v>1928</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E40" s="4">
+        <v>32</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G40" s="4">
+        <v>68</v>
+      </c>
+      <c r="H40" s="5"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="7">
+        <v>46314</v>
+      </c>
+      <c r="C41" s="2">
+        <v>1928</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41" s="2">
+        <v>43</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="G41" s="2">
+        <v>57</v>
+      </c>
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" s="11"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="11"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="11"/>
+      <c r="H42" s="13"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" s="2"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="4"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="5"/>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="2"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="4"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="5"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" s="2"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="4"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="5"/>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" s="2"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="3"/>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="4"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="5"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="2"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="3"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="4"/>
+      <c r="B52" s="8"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="5"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="2"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="3"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" s="4"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="5"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" s="2"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="3"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" s="11"/>
+      <c r="B56" s="12"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="13"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="2"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="3"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" s="4"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="5"/>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="2"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="3"/>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="4"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="5"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="2"/>
+      <c r="B61" s="7"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="3"/>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" s="4"/>
+      <c r="B62" s="8"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" s="2"/>
+      <c r="B63" s="7"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="3"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" s="4"/>
+      <c r="B64" s="8"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="5"/>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A65" s="2"/>
+      <c r="B65" s="7"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+      <c r="G65" s="2"/>
+      <c r="H65" s="3"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A66" s="4"/>
+      <c r="B66" s="8"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+      <c r="G66" s="4"/>
+      <c r="H66" s="5"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A67" s="2"/>
+      <c r="B67" s="7"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
+      <c r="F67" s="2"/>
+      <c r="G67" s="2"/>
+      <c r="H67" s="3"/>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A68" s="4"/>
+      <c r="B68" s="8"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
+      <c r="G68" s="4"/>
+      <c r="H68" s="5"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A69" s="2"/>
+      <c r="B69" s="7"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
+      <c r="F69" s="2"/>
+      <c r="G69" s="2"/>
+      <c r="H69" s="3"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A70" s="11"/>
+      <c r="B70" s="12"/>
+      <c r="C70" s="11"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="11"/>
+      <c r="F70" s="11"/>
+      <c r="G70" s="11"/>
+      <c r="H70" s="13"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A71" s="2"/>
+      <c r="B71" s="7"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
+      <c r="H71" s="3"/>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A72" s="4"/>
+      <c r="B72" s="8"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+      <c r="H72" s="5"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A73" s="2"/>
+      <c r="B73" s="7"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="2"/>
+      <c r="E73" s="2"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
+      <c r="H73" s="3"/>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A74" s="4"/>
+      <c r="B74" s="8"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4"/>
+      <c r="F74" s="4"/>
+      <c r="G74" s="4"/>
+      <c r="H74" s="5"/>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A75" s="2"/>
+      <c r="B75" s="7"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="E75" s="2"/>
+      <c r="F75" s="2"/>
+      <c r="G75" s="2"/>
+      <c r="H75" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2422,7 +4091,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2507,7 +4176,7 @@
       <c r="G3">
         <v>4</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>16</v>
       </c>
       <c r="J3">
@@ -2621,7 +4290,7 @@
       <c r="G6">
         <v>3.5</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>16</v>
       </c>
       <c r="J6">
@@ -2659,7 +4328,7 @@
       <c r="G7">
         <v>4</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>14.5</v>
       </c>
       <c r="J7">
@@ -2718,7 +4387,7 @@
         <v>1500</v>
       </c>
       <c r="D9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E9">
         <v>13</v>
@@ -2729,7 +4398,7 @@
       <c r="G9">
         <v>4</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>14</v>
       </c>
       <c r="J9">
@@ -2764,7 +4433,7 @@
       <c r="G10">
         <v>3</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>14</v>
       </c>
       <c r="J10">
@@ -2834,7 +4503,7 @@
       <c r="G12">
         <v>3</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>15</v>
       </c>
       <c r="J12">
@@ -2869,7 +4538,7 @@
       <c r="G13">
         <v>4</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>14</v>
       </c>
       <c r="J13">
@@ -2907,7 +4576,7 @@
       <c r="G14">
         <v>3.5</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>15</v>
       </c>
       <c r="J14">
@@ -2983,7 +4652,7 @@
       <c r="G16">
         <v>3</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <v>15</v>
       </c>
       <c r="J16">
@@ -3059,7 +4728,7 @@
       <c r="G18">
         <v>4</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <v>15</v>
       </c>
       <c r="J18">
@@ -3097,7 +4766,7 @@
       <c r="G19">
         <v>3</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <v>16</v>
       </c>
       <c r="J19">
@@ -3167,7 +4836,7 @@
       <c r="G21">
         <v>5</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>16</v>
       </c>
       <c r="J21">
@@ -3202,7 +4871,7 @@
       <c r="G22">
         <v>5</v>
       </c>
-      <c r="H22">
+      <c r="I22">
         <v>16</v>
       </c>
       <c r="J22">
@@ -3237,7 +4906,7 @@
       <c r="G23">
         <v>3.5</v>
       </c>
-      <c r="H23">
+      <c r="I23">
         <v>13.5</v>
       </c>
       <c r="J23">
@@ -3340,7 +5009,7 @@
         <v>1764</v>
       </c>
       <c r="D26" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E26">
         <v>17</v>
@@ -3351,7 +5020,7 @@
       <c r="G26">
         <v>3</v>
       </c>
-      <c r="H26">
+      <c r="I26">
         <v>15</v>
       </c>
       <c r="J26">
@@ -3410,7 +5079,7 @@
         <v>1764</v>
       </c>
       <c r="D28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E28">
         <v>17</v>
@@ -3421,7 +5090,7 @@
       <c r="G28">
         <v>4</v>
       </c>
-      <c r="H28">
+      <c r="I28">
         <v>14</v>
       </c>
       <c r="J28">
@@ -3456,7 +5125,7 @@
       <c r="G29">
         <v>3</v>
       </c>
-      <c r="H29">
+      <c r="I29">
         <v>14</v>
       </c>
       <c r="J29">
@@ -3480,7 +5149,7 @@
         <v>1598</v>
       </c>
       <c r="D30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E30">
         <v>18</v>
@@ -3512,7 +5181,7 @@
         <v>1598</v>
       </c>
       <c r="D31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E31">
         <v>18.5</v>
@@ -3520,7 +5189,7 @@
       <c r="F31">
         <v>17</v>
       </c>
-      <c r="H31">
+      <c r="I31">
         <v>15</v>
       </c>
       <c r="J31">
@@ -3544,7 +5213,7 @@
         <v>1598</v>
       </c>
       <c r="D32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E32">
         <v>19</v>
@@ -3576,7 +5245,7 @@
         <v>1598</v>
       </c>
       <c r="D33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E33">
         <v>17</v>
@@ -3602,7 +5271,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B34" s="7">
         <v>46227</v>
@@ -3622,7 +5291,7 @@
       <c r="G34">
         <v>3.1</v>
       </c>
-      <c r="H34">
+      <c r="I34">
         <v>13.8</v>
       </c>
       <c r="J34">
@@ -3635,7 +5304,7 @@
         <v>4.2</v>
       </c>
       <c r="M34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
@@ -3660,7 +5329,7 @@
       <c r="G35">
         <v>4</v>
       </c>
-      <c r="H35">
+      <c r="I35">
         <v>14</v>
       </c>
       <c r="J35">
@@ -3684,7 +5353,7 @@
         <v>1500</v>
       </c>
       <c r="D36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E36">
         <v>16.5</v>
@@ -3719,7 +5388,7 @@
         <v>1500</v>
       </c>
       <c r="D37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E37">
         <v>17</v>
@@ -3730,7 +5399,7 @@
       <c r="G37">
         <v>5.5</v>
       </c>
-      <c r="H37">
+      <c r="I37">
         <v>15.5</v>
       </c>
       <c r="J37">
@@ -3754,7 +5423,7 @@
         <v>1500</v>
       </c>
       <c r="D38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E38">
         <v>15</v>
@@ -3783,7 +5452,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B39" s="7">
         <v>46266</v>
@@ -3803,7 +5472,7 @@
       <c r="G39">
         <v>2.5</v>
       </c>
-      <c r="H39">
+      <c r="I39">
         <v>13.5</v>
       </c>
       <c r="J39">
@@ -3816,7 +5485,7 @@
         <v>4</v>
       </c>
       <c r="M39" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.2">
@@ -3865,7 +5534,7 @@
         <v>929</v>
       </c>
       <c r="D41" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E41">
         <v>17</v>
@@ -3938,7 +5607,7 @@
         <v>948</v>
       </c>
       <c r="D43" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E43">
         <v>15</v>
@@ -3976,7 +5645,7 @@
         <v>13060</v>
       </c>
       <c r="D44" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E44">
         <v>15.5</v>
@@ -4049,7 +5718,7 @@
         <v>2052</v>
       </c>
       <c r="D46" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E46">
         <v>16</v>
@@ -4146,7 +5815,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>17</v>
       </c>
@@ -4157,7 +5826,7 @@
         <v>2052</v>
       </c>
       <c r="D49" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E49">
         <v>17</v>
@@ -4181,15 +5850,1151 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A50" s="2" t="s">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B50" s="8">
+        <v>46281</v>
+      </c>
+      <c r="C50" s="4">
+        <v>1943</v>
+      </c>
+      <c r="D50" t="s">
+        <v>60</v>
+      </c>
+      <c r="E50">
+        <v>19.8</v>
+      </c>
+      <c r="F50">
+        <v>14</v>
+      </c>
+      <c r="G50">
+        <v>2.6</v>
+      </c>
+      <c r="I50">
+        <v>13.4</v>
+      </c>
+      <c r="J50">
+        <v>9.5</v>
+      </c>
+      <c r="K50">
+        <v>31</v>
+      </c>
+      <c r="L50">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A51" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B51" s="8">
+        <v>46281</v>
+      </c>
+      <c r="C51" s="4">
+        <v>1943</v>
+      </c>
+      <c r="D51" t="s">
+        <v>61</v>
+      </c>
+      <c r="E51">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="F51">
+        <v>7.4</v>
+      </c>
+      <c r="G51">
+        <v>3</v>
+      </c>
+      <c r="H51">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="J51">
+        <v>7.6</v>
+      </c>
+      <c r="K51">
+        <v>30.2</v>
+      </c>
+      <c r="M51" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B50" s="7">
+      <c r="B52" s="7">
+        <v>46289</v>
+      </c>
+      <c r="C52" s="2">
+        <v>1974</v>
+      </c>
+      <c r="D52" t="s">
+        <v>87</v>
+      </c>
+      <c r="E52">
+        <v>17</v>
+      </c>
+      <c r="F52">
+        <v>10</v>
+      </c>
+      <c r="G52">
+        <v>3</v>
+      </c>
+      <c r="H52">
+        <v>13</v>
+      </c>
+      <c r="I52">
+        <v>5</v>
+      </c>
+      <c r="J52">
+        <v>7</v>
+      </c>
+      <c r="K52">
+        <v>35</v>
+      </c>
+      <c r="L52">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B53" s="7">
+        <v>46289</v>
+      </c>
+      <c r="C53" s="2">
+        <v>1974</v>
+      </c>
+      <c r="D53" t="s">
+        <v>60</v>
+      </c>
+      <c r="E53">
+        <v>17</v>
+      </c>
+      <c r="F53">
+        <v>11</v>
+      </c>
+      <c r="G53">
+        <v>3</v>
+      </c>
+      <c r="I53">
+        <v>12</v>
+      </c>
+      <c r="J53">
+        <v>10</v>
+      </c>
+      <c r="K53">
+        <v>36</v>
+      </c>
+      <c r="L53">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B54" s="7">
+        <v>46289</v>
+      </c>
+      <c r="C54" s="2">
+        <v>1974</v>
+      </c>
+      <c r="D54" t="s">
+        <v>68</v>
+      </c>
+      <c r="E54">
+        <v>18</v>
+      </c>
+      <c r="F54">
+        <v>7</v>
+      </c>
+      <c r="G54">
+        <v>4</v>
+      </c>
+      <c r="H54">
+        <v>16</v>
+      </c>
+      <c r="J54">
+        <v>9</v>
+      </c>
+      <c r="K54">
+        <v>35</v>
+      </c>
+      <c r="L54">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B55" s="7">
+        <v>46289</v>
+      </c>
+      <c r="C55" s="2">
+        <v>1974</v>
+      </c>
+      <c r="D55" t="s">
+        <v>72</v>
+      </c>
+      <c r="E55">
+        <v>17</v>
+      </c>
+      <c r="F55">
+        <v>8</v>
+      </c>
+      <c r="G55">
+        <v>5</v>
+      </c>
+      <c r="I55">
+        <v>13</v>
+      </c>
+      <c r="J55">
+        <v>10</v>
+      </c>
+      <c r="K55">
+        <v>36</v>
+      </c>
+      <c r="L55">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B56" s="8">
         <v>46275</v>
       </c>
-      <c r="C50" s="2">
-        <v>2052</v>
+      <c r="C56" s="4">
+        <v>935</v>
+      </c>
+      <c r="D56" t="s">
+        <v>61</v>
+      </c>
+      <c r="E56">
+        <v>16</v>
+      </c>
+      <c r="F56">
+        <v>7</v>
+      </c>
+      <c r="G56">
+        <v>3</v>
+      </c>
+      <c r="H56">
+        <v>16</v>
+      </c>
+      <c r="J56">
+        <v>7</v>
+      </c>
+      <c r="K56">
+        <v>32</v>
+      </c>
+      <c r="L56">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B57" s="8">
+        <v>46275</v>
+      </c>
+      <c r="C57" s="4">
+        <v>935</v>
+      </c>
+      <c r="D57" t="s">
+        <v>89</v>
+      </c>
+      <c r="E57">
+        <v>17</v>
+      </c>
+      <c r="F57">
+        <v>3</v>
+      </c>
+      <c r="G57">
+        <v>3</v>
+      </c>
+      <c r="H57">
+        <v>16</v>
+      </c>
+      <c r="J57">
+        <v>7</v>
+      </c>
+      <c r="K57">
+        <v>33</v>
+      </c>
+      <c r="L57">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" s="7">
+        <v>46294</v>
+      </c>
+      <c r="C58" s="2">
+        <v>1527</v>
+      </c>
+      <c r="D58" t="s">
+        <v>87</v>
+      </c>
+      <c r="E58">
+        <v>15</v>
+      </c>
+      <c r="F58">
+        <v>11</v>
+      </c>
+      <c r="G58">
+        <v>3</v>
+      </c>
+      <c r="H58">
+        <v>16</v>
+      </c>
+      <c r="I58">
+        <v>8</v>
+      </c>
+      <c r="J58">
+        <v>7</v>
+      </c>
+      <c r="K58">
+        <v>32</v>
+      </c>
+      <c r="L58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B59" s="7">
+        <v>46294</v>
+      </c>
+      <c r="C59" s="2">
+        <v>1527</v>
+      </c>
+      <c r="D59" t="s">
+        <v>60</v>
+      </c>
+      <c r="E59">
+        <v>15</v>
+      </c>
+      <c r="F59">
+        <v>13</v>
+      </c>
+      <c r="G59">
+        <v>4</v>
+      </c>
+      <c r="I59">
+        <v>15</v>
+      </c>
+      <c r="J59">
+        <v>10</v>
+      </c>
+      <c r="K59">
+        <v>34</v>
+      </c>
+      <c r="L59">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60" s="7">
+        <v>46294</v>
+      </c>
+      <c r="C60" s="2">
+        <v>1527</v>
+      </c>
+      <c r="D60" t="s">
+        <v>91</v>
+      </c>
+      <c r="E60">
+        <v>16</v>
+      </c>
+      <c r="F60">
+        <v>3</v>
+      </c>
+      <c r="G60">
+        <v>5</v>
+      </c>
+      <c r="H60">
+        <v>23</v>
+      </c>
+      <c r="J60">
+        <v>8</v>
+      </c>
+      <c r="K60">
+        <v>35</v>
+      </c>
+      <c r="L60">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B61" s="7">
+        <v>46294</v>
+      </c>
+      <c r="C61" s="2">
+        <v>1527</v>
+      </c>
+      <c r="D61" t="s">
+        <v>90</v>
+      </c>
+      <c r="E61">
+        <v>17</v>
+      </c>
+      <c r="F61">
+        <v>4</v>
+      </c>
+      <c r="G61">
+        <v>5.5</v>
+      </c>
+      <c r="I61">
+        <v>17</v>
+      </c>
+      <c r="J61">
+        <v>11</v>
+      </c>
+      <c r="K61">
+        <v>36</v>
+      </c>
+      <c r="L61">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B62" s="7">
+        <v>46294</v>
+      </c>
+      <c r="C62" s="2">
+        <v>1527</v>
+      </c>
+      <c r="D62" t="s">
+        <v>61</v>
+      </c>
+      <c r="E62">
+        <v>16</v>
+      </c>
+      <c r="F62">
+        <v>8</v>
+      </c>
+      <c r="G62">
+        <v>5</v>
+      </c>
+      <c r="H62">
+        <v>22</v>
+      </c>
+      <c r="J62">
+        <v>7</v>
+      </c>
+      <c r="K62">
+        <v>34</v>
+      </c>
+      <c r="L62">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B63" s="9">
+        <v>46276</v>
+      </c>
+      <c r="C63" s="2">
+        <v>1548</v>
+      </c>
+      <c r="D63" t="s">
+        <v>84</v>
+      </c>
+      <c r="E63">
+        <v>17</v>
+      </c>
+      <c r="F63">
+        <v>9</v>
+      </c>
+      <c r="G63">
+        <v>3</v>
+      </c>
+      <c r="H63">
+        <v>14</v>
+      </c>
+      <c r="I63">
+        <v>7</v>
+      </c>
+      <c r="J63">
+        <v>6.5</v>
+      </c>
+      <c r="K63">
+        <v>35</v>
+      </c>
+      <c r="L63">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A64" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B64" s="8">
+        <v>46303</v>
+      </c>
+      <c r="C64" s="4">
+        <v>2004</v>
+      </c>
+      <c r="D64" t="s">
+        <v>60</v>
+      </c>
+      <c r="E64">
+        <v>18</v>
+      </c>
+      <c r="F64">
+        <v>11</v>
+      </c>
+      <c r="G64">
+        <v>3</v>
+      </c>
+      <c r="I64">
+        <v>12</v>
+      </c>
+      <c r="J64">
+        <v>10</v>
+      </c>
+      <c r="K64">
+        <v>36</v>
+      </c>
+      <c r="L64">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A65" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B65" s="8">
+        <v>46303</v>
+      </c>
+      <c r="C65" s="4">
+        <v>2004</v>
+      </c>
+      <c r="D65" t="s">
+        <v>87</v>
+      </c>
+      <c r="E65">
+        <v>18</v>
+      </c>
+      <c r="F65">
+        <v>10</v>
+      </c>
+      <c r="G65">
+        <v>2</v>
+      </c>
+      <c r="H65">
+        <v>13</v>
+      </c>
+      <c r="I65">
+        <v>5</v>
+      </c>
+      <c r="J65">
+        <v>7</v>
+      </c>
+      <c r="K65">
+        <v>35</v>
+      </c>
+      <c r="L65">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B66" s="7">
+        <v>46302</v>
+      </c>
+      <c r="C66" s="2">
+        <v>7374</v>
+      </c>
+      <c r="D66" t="s">
+        <v>60</v>
+      </c>
+      <c r="E66">
+        <v>18.5</v>
+      </c>
+      <c r="F66">
+        <v>10.5</v>
+      </c>
+      <c r="G66">
+        <v>3.5</v>
+      </c>
+      <c r="I66">
+        <v>11</v>
+      </c>
+      <c r="J66">
+        <v>9</v>
+      </c>
+      <c r="K66">
+        <v>38</v>
+      </c>
+      <c r="L66">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A67" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B67" s="8">
+        <v>46309</v>
+      </c>
+      <c r="C67" s="4">
+        <v>1390</v>
+      </c>
+      <c r="D67" t="s">
+        <v>84</v>
+      </c>
+      <c r="E67">
+        <v>16</v>
+      </c>
+      <c r="F67">
+        <v>14</v>
+      </c>
+      <c r="G67">
+        <v>2</v>
+      </c>
+      <c r="H67">
+        <v>14</v>
+      </c>
+      <c r="I67">
+        <v>6</v>
+      </c>
+      <c r="J67">
+        <v>6.5</v>
+      </c>
+      <c r="K67">
+        <v>34</v>
+      </c>
+      <c r="L67">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A68" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B68" s="8">
+        <v>46309</v>
+      </c>
+      <c r="C68" s="4">
+        <v>1390</v>
+      </c>
+      <c r="D68" t="s">
+        <v>44</v>
+      </c>
+      <c r="E68">
+        <v>17</v>
+      </c>
+      <c r="F68">
+        <v>16</v>
+      </c>
+      <c r="G68">
+        <v>2.5</v>
+      </c>
+      <c r="I68">
+        <v>13</v>
+      </c>
+      <c r="J68">
+        <v>8</v>
+      </c>
+      <c r="K68">
+        <v>36</v>
+      </c>
+      <c r="L68">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B69" s="7">
+        <v>46309</v>
+      </c>
+      <c r="C69" s="2">
+        <v>978</v>
+      </c>
+      <c r="D69" t="s">
+        <v>44</v>
+      </c>
+      <c r="E69">
+        <v>15</v>
+      </c>
+      <c r="F69">
+        <v>16</v>
+      </c>
+      <c r="G69">
+        <v>3</v>
+      </c>
+      <c r="I69">
+        <v>11</v>
+      </c>
+      <c r="J69">
+        <v>9</v>
+      </c>
+      <c r="K69">
+        <v>37</v>
+      </c>
+      <c r="L69">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B70" s="7">
+        <v>46309</v>
+      </c>
+      <c r="C70" s="2">
+        <v>978</v>
+      </c>
+      <c r="D70" t="s">
+        <v>84</v>
+      </c>
+      <c r="E70">
+        <v>14</v>
+      </c>
+      <c r="F70">
+        <v>13</v>
+      </c>
+      <c r="G70">
+        <v>3</v>
+      </c>
+      <c r="H70">
+        <v>12</v>
+      </c>
+      <c r="I70">
+        <v>7</v>
+      </c>
+      <c r="J70">
+        <v>7</v>
+      </c>
+      <c r="K70">
+        <v>35</v>
+      </c>
+      <c r="L70">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A71" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B71" s="9">
+        <v>46309</v>
+      </c>
+      <c r="C71" s="17">
+        <v>978</v>
+      </c>
+      <c r="D71" t="s">
+        <v>84</v>
+      </c>
+      <c r="E71">
+        <v>15</v>
+      </c>
+      <c r="F71">
+        <v>13</v>
+      </c>
+      <c r="G71">
+        <v>2</v>
+      </c>
+      <c r="H71">
+        <v>12</v>
+      </c>
+      <c r="I71">
+        <v>5</v>
+      </c>
+      <c r="J71">
+        <v>6</v>
+      </c>
+      <c r="K71">
+        <v>35</v>
+      </c>
+      <c r="L71">
+        <v>5</v>
+      </c>
+      <c r="M71" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A72" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B72" s="8">
+        <v>46310</v>
+      </c>
+      <c r="C72" s="4">
+        <v>1094</v>
+      </c>
+      <c r="D72" t="s">
+        <v>44</v>
+      </c>
+      <c r="E72">
+        <v>15</v>
+      </c>
+      <c r="F72">
+        <v>14</v>
+      </c>
+      <c r="G72">
+        <v>6</v>
+      </c>
+      <c r="I72">
+        <v>10</v>
+      </c>
+      <c r="J72">
+        <v>9</v>
+      </c>
+      <c r="K72">
+        <v>37</v>
+      </c>
+      <c r="L72">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A73" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B73" s="8">
+        <v>46310</v>
+      </c>
+      <c r="C73" s="4">
+        <v>1094</v>
+      </c>
+      <c r="D73" t="s">
+        <v>84</v>
+      </c>
+      <c r="E73">
+        <v>15</v>
+      </c>
+      <c r="F73">
+        <v>12</v>
+      </c>
+      <c r="G73">
+        <v>6</v>
+      </c>
+      <c r="H73">
+        <v>10</v>
+      </c>
+      <c r="I73">
+        <v>6</v>
+      </c>
+      <c r="J73">
+        <v>6</v>
+      </c>
+      <c r="K73">
+        <v>36</v>
+      </c>
+      <c r="L73">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B74" s="7">
+        <v>46311</v>
+      </c>
+      <c r="C74" s="2">
+        <v>1701</v>
+      </c>
+      <c r="D74" t="s">
+        <v>44</v>
+      </c>
+      <c r="E74">
+        <v>16</v>
+      </c>
+      <c r="F74">
+        <v>16.5</v>
+      </c>
+      <c r="G74">
+        <v>2.5</v>
+      </c>
+      <c r="I74">
+        <v>10.5</v>
+      </c>
+      <c r="J74">
+        <v>9.5</v>
+      </c>
+      <c r="K74">
+        <v>33.5</v>
+      </c>
+      <c r="L74">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B75" s="7">
+        <v>46311</v>
+      </c>
+      <c r="C75" s="2">
+        <v>1701</v>
+      </c>
+      <c r="D75" t="s">
+        <v>84</v>
+      </c>
+      <c r="E75">
+        <v>15.5</v>
+      </c>
+      <c r="F75">
+        <v>15.5</v>
+      </c>
+      <c r="G75">
+        <v>2.5</v>
+      </c>
+      <c r="H75">
+        <v>13.5</v>
+      </c>
+      <c r="I75">
+        <v>4.5</v>
+      </c>
+      <c r="J75">
+        <v>7.5</v>
+      </c>
+      <c r="K75">
+        <v>32.5</v>
+      </c>
+      <c r="L75">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A76" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B76" s="8">
+        <v>46310</v>
+      </c>
+      <c r="C76" s="4">
+        <v>1187</v>
+      </c>
+      <c r="D76" t="s">
+        <v>44</v>
+      </c>
+      <c r="E76">
+        <v>20</v>
+      </c>
+      <c r="F76">
+        <v>13.5</v>
+      </c>
+      <c r="G76">
+        <v>2</v>
+      </c>
+      <c r="I76">
+        <v>17</v>
+      </c>
+      <c r="K76">
+        <v>35.5</v>
+      </c>
+      <c r="L76">
+        <v>5.5</v>
+      </c>
+      <c r="M76" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A77" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B77" s="8">
+        <v>46310</v>
+      </c>
+      <c r="C77" s="4">
+        <v>1187</v>
+      </c>
+      <c r="D77" t="s">
+        <v>100</v>
+      </c>
+      <c r="E77">
+        <v>20</v>
+      </c>
+      <c r="F77">
+        <v>16</v>
+      </c>
+      <c r="G77">
+        <v>2</v>
+      </c>
+      <c r="J77">
+        <v>17.5</v>
+      </c>
+      <c r="K77">
+        <v>34.5</v>
+      </c>
+      <c r="L77">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B78" s="7">
+        <v>46314</v>
+      </c>
+      <c r="C78" s="2">
+        <v>1928</v>
+      </c>
+      <c r="D78" t="s">
+        <v>84</v>
+      </c>
+      <c r="E78">
+        <v>16.5</v>
+      </c>
+      <c r="F78">
+        <v>13.5</v>
+      </c>
+      <c r="G78">
+        <v>3</v>
+      </c>
+      <c r="H78">
+        <v>12</v>
+      </c>
+      <c r="I78">
+        <v>5</v>
+      </c>
+      <c r="J78">
+        <v>5</v>
+      </c>
+      <c r="K78">
+        <v>36</v>
+      </c>
+      <c r="L78">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B79" s="7">
+        <v>46314</v>
+      </c>
+      <c r="C79" s="2">
+        <v>1928</v>
+      </c>
+      <c r="D79" t="s">
+        <v>44</v>
+      </c>
+      <c r="E79">
+        <v>16</v>
+      </c>
+      <c r="F79">
+        <v>16</v>
+      </c>
+      <c r="G79">
+        <v>3</v>
+      </c>
+      <c r="I79">
+        <v>13</v>
+      </c>
+      <c r="J79">
+        <v>7</v>
+      </c>
+      <c r="K79">
+        <v>38</v>
+      </c>
+      <c r="L79">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B80" s="7">
+        <v>46314</v>
+      </c>
+      <c r="C80" s="2">
+        <v>1928</v>
+      </c>
+      <c r="D80" t="s">
+        <v>101</v>
+      </c>
+      <c r="E80">
+        <v>18</v>
+      </c>
+      <c r="F80">
+        <v>16</v>
+      </c>
+      <c r="H80">
+        <v>16</v>
+      </c>
+      <c r="J80">
+        <v>6.5</v>
+      </c>
+      <c r="K80">
+        <v>37</v>
+      </c>
+      <c r="L80">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B81" s="7">
+        <v>46314</v>
+      </c>
+      <c r="C81" s="2">
+        <v>1928</v>
+      </c>
+      <c r="D81" t="s">
+        <v>102</v>
+      </c>
+      <c r="E81">
+        <v>15.5</v>
+      </c>
+      <c r="F81">
+        <v>13</v>
+      </c>
+      <c r="G81">
+        <v>3</v>
+      </c>
+      <c r="H81">
+        <v>13</v>
+      </c>
+      <c r="J81">
+        <v>7</v>
+      </c>
+      <c r="K81">
+        <v>36</v>
+      </c>
+      <c r="L81">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>